<commit_message>
feat(F-NAR-019): ATOM-AUT.RAN.001-08 Le pont de Nino
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.RAN.001-08.xlsx
+++ b/stories/arbres/ATOM-AUT.RAN.001-08.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nino veut s'asseoir dans le t-shirt chaud, avec la petite voiture qui a passé sous le pont. L'arche s'écroule sur la voiture. Il cherche, met les cubes dans la caisse. La voiture apparaît. Canapé, linge chaud.</t>
+          <t>L'odeur de citron arrive avant le sol sec. Sur un carreau mouillé, un éclat de citron brille. Nino veut le pont du tapis, maintenant, pour la voiture jusqu'au canapé, puis le t-shirt chaud. Un cube glisse : l'arche s'écroule sur la voiture. Il cherche dans le linge, sous le canapé, puis prend toute la pile : les cubes s'éparpillent. Il refuse de foncer, pose un cube, retrouve la voiture. Sur le carreau libre, l'éclat de citron tient.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le carrelage sent encore le citron. Papa vient de passer la serpillière. Les carreaux sont un peu frais. Puis le tapis du salon est épais. Ça sent le propre. Oui, tout propre. Près du canapé, une pile de linge attend. Un petit t-shirt est encore chaud. En ce moment, Nino est au milieu du tapis. Il a des cubes. Il construit un pont. Les cubes tapent. C'est un pont, papa. Un pont bien solide ? Oui, il est solide. Il va jusqu'où, ton pont ? Jusqu'au canapé, maman. Nino pose encore un cube. Clic. Il pose un cube à gauche. Puis un cube à droite. Le pont a une arche. Je vois l'arche, Nino. Une petite voiture peut passer. On essaie. Nino prend une petite voiture. Il la pousse vers l'arche. Un cube glisse. L'arche a un trou. La voiture bute. Oh, elle ne passe pas. Le cube est tombé. Nino repose le cube. Clic. L'arche est ronde, encore. La voiture passe dessous. Elle est passée ! Elle rentre à la maison ? Oui, puis on s'assoit. Nino veut le t-shirt chaud. Il pousse encore la voiture. Trois cubes tombent d'un coup. L'arche s'écroule sur la voiture. Oh. Le pont est tombé. Où est ma petite voiture ? Dans la pile de linge ? Nino fouille le t-shirt chaud. Le tissu sent le savon. Pas de voiture. Sous le canapé ? Il se penche. De la poussière, un fil. Elle est perdue. Les cubes sont encore au milieu. Je veux voir dessous. Nino prend un cube. Il le pose dans la caisse. Toc. La caisse sent le bois.</t>
+          <t>L'odeur de citron arrive avant le sol sec. Papa tord la serpillière au-dessus du seau. Le seau fait un petit plouf. Ça sent le propre. Oui, le citron a fini. Sur un carreau mouillé, un éclat de citron brille. Il est jaune, papa. C'est le citron, sur le carreau. Les carreaux sont un peu frais. Puis le tapis du salon est épais. Le sol est propre, Nino. Tu restes sur le tapis ? Oui, le sol est mouillé. Près du canapé, une pile de linge attend. Un petit t-shirt reste chaud, au sommet. Je veux mon pont, maintenant ! Pendant que le sol sèche ? Oui, un pont jusqu'au canapé. En ce moment, Nino saisit un cube. Le cube bleu pèse un peu, dans sa main. Il pose le cube sur le tapis épais. Le bois tape, un petit clic. C'est le pont du tapis. Un pont bien solide ? Oui, il est solide. Il va jusqu'où, ton pont ? Jusqu'au canapé, maman. Nino pose un cube à gauche. Puis un cube à droite. Le pont a une arche. Je vois l'arche, Nino. Une petite voiture peut passer. On essaie ? La petite voiture rouge attend près du tapis. Toi, tu vas sous le pont. Nino la pousse vers l'arche. Un cube glisse. L'arche a un trou. Oh, elle ne passe pas. Le cube est tombé. Nino repose le cube, trop vite. Le cube penche, de travers. La voiture bute, une seconde fois. Ça ne veut pas ! Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu regardes le cube, d'abord ? Oui, maman. Il pose le cube, sans se presser. L'arche redevient ronde. La voiture passe dessous. Elle est passée ! Elle rentre à la maison ? Oui, puis on s'assoit. Nino veut le t-shirt chaud. Maintenant, le t-shirt ! Il pousse la voiture trop fort. Trois cubes tombent d'un coup. L'arche s'écroule sur la voiture. Oh. Le pont est tombé. Où est ma petite voiture ? Dans la pile de linge ? Nino fouille le t-shirt chaud. Le tissu sent le savon. Pas de voiture. Sous le canapé ? Il se penche. De la poussière, un fil. Elle est perdue. L'éclat de citron tremble, sur le carreau. Je prends tout, d'un coup ! Il saisit la pile trop vite. Les cubes glissent entre ses doigts. Le tapis disparaît sous les cubes. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous les cubes ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le carrelage sent encore le citron. Papa vient de passer la serpillière. Les carreaux sont un peu frais. Puis le tapis du salon est épais. Ça sent le propre. Oui, tout propre. Près du canapé, une pile de linge attend. Un petit t-shirt est encore chaud. En ce moment, Nino est au milieu du tapis. Il a des cubes. Il construit un pont. Les cubes tapent. C'est un pont, papa. Un pont bien solide ? Oui, il est solide. Il va jusqu'où, ton pont ? Jusqu'au canapé, maman. Nino pose encore un cube. Clic. Il pose un cube à gauche. Puis un cube à droite. Le pont a une arche. Je vois l'arche, Nino. Une petite voiture peut passer. On essaie. Nino prend une petite voiture. Il la pousse vers l'arche. Un cube glisse. L'arche a un trou. La voiture bute. Oh, elle ne passe pas. Le cube est tombé. Nino repose le cube. Clic. L'arche est ronde, encore. La voiture passe dessous. Elle est passée ! Elle rentre à la maison ? Oui, puis on s'assoit. Nino veut le t-shirt chaud. Il pousse encore la voiture. Trois cubes tombent d'un coup. L'arche s'écroule sur la voiture. Oh. Le pont est tombé. Où est ma petite voiture ? Dans la pile de linge ? Nino fouille le t-shirt chaud. Le tissu sent le savon. Pas de voiture. Sous le canapé ? Il se penche. De la poussière, un fil. Elle est perdue. Les cubes sont encore au milieu. Je veux voir dessous. Nino prend un cube. Il le pose dans la caisse. Toc. La caisse sent le bois.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'odeur de citron arrive avant le sol sec. Papa tord la serpillière au-dessus du seau. Le seau fait un petit plouf. Ça sent le propre. Oui, le citron a fini. Sur un carreau mouillé, un &lt;emphasis level="moderate"&gt;éclat de citron&lt;/emphasis&gt; brille. Il est jaune, papa. C'est le citron, sur le carreau. Les carreaux sont un peu frais. Puis le tapis du salon est épais. Le sol est propre, Nino. Tu restes sur le tapis ? Oui, le sol est mouillé. Près du canapé, une pile de linge attend. Un petit t-shirt reste chaud, au sommet. Je veux mon pont, maintenant ! Pendant que le sol sèche ? Oui, un pont jusqu'au canapé. En ce moment, Nino saisit un cube. Le cube bleu pèse un peu, dans sa main. Il pose le cube sur le tapis épais. Le bois tape, un petit clic. C'est le pont du tapis. Un pont bien solide ? Oui, il est solide. Il va jusqu'où, ton pont ? Jusqu'au canapé, maman. Nino pose un cube à gauche. Puis un cube à droite. Le pont a une arche. Je vois l'arche, Nino. Une petite voiture peut passer. On essaie ? La petite voiture rouge attend près du tapis. Toi, tu vas sous le pont. Nino la pousse vers l'arche. Un cube glisse. L'arche a un trou. Oh, elle ne passe pas. Le cube est tombé. Nino repose le cube, trop vite. Le cube penche, de travers. La voiture bute, une seconde fois. Ça ne veut pas ! Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu regardes le cube, d'abord ? Oui, maman. Il pose le cube, sans se presser. L'arche redevient ronde. La voiture passe dessous. Elle est passée ! Elle rentre à la maison ? Oui, puis on s'assoit. Nino veut le t-shirt chaud. Maintenant, le t-shirt ! Il pousse la voiture trop fort. Trois cubes tombent d'un coup. L'arche s'écroule sur la voiture. Oh. Le pont est tombé. Où est ma petite voiture ? Dans la pile de linge ? Nino fouille le t-shirt chaud. Le tissu sent le savon. Pas de voiture. Sous le canapé ? Il se penche. De la poussière, un fil. Elle est perdue. L'éclat de citron tremble, sur le carreau. Je prends tout, d'un coup ! Il saisit la pile trop vite. Les cubes glissent entre ses doigts. Le tapis disparaît sous les cubes. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous les cubes ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Martial joue dans le salon. Papa plie le linge. Martial a des cubes. Il construit un pont. Les cubes tapent. Puis le jeu est fini. Papa dit : c'est l'heure de &lt;emphasis&gt;ranger&lt;/emphasis&gt;. Ranger, c'est remettre. Martial prend un cube. Il le met dans la caisse. Il prend un autre cube. Il le met dans la caisse. La caisse sent le bois. Plus tard, Martial sort des voitures. Il les fait rouler. Le jeu se termine encore. Martial se souvient. Il range. Les voitures vont dans la caisse. Le tapis redevient libre. Papa dit : après le jeu, on range. Les jouets retournent dans la caisse. Martial ferme le couvercle. Ça fait toc. [pause]</t>
+          <t>L'odeur de citron arrive avant le sol sec. Papa tord la serpillière au-dessus du seau. Le seau fait un petit plouf. Ça sent le propre. Oui, le citron a fini. Sur un carreau mouillé, un &lt;emphasis&gt;éclat de citron&lt;/emphasis&gt; brille. Il est jaune, papa. C'est le citron, sur le carreau. Les carreaux sont un peu frais. Puis le tapis du salon est épais. Le sol est propre, Nino. Tu restes sur le tapis ? Oui, le sol est mouillé. Près du canapé, une pile de linge attend. Un petit t-shirt reste chaud, au sommet. Je veux mon pont, maintenant ! Pendant que le sol sèche ? Oui, un pont jusqu'au canapé. En ce moment, Nino saisit un cube. Le cube bleu pèse un peu, dans sa main. Il pose le cube sur le tapis épais. Le bois tape, un petit clic. C'est le pont du tapis. Un pont bien solide ? Oui, il est solide. Il va jusqu'où, ton pont ? Jusqu'au canapé, maman. Nino pose un cube à gauche. Puis un cube à droite. Le pont a une arche. Je vois l'arche, Nino. Une petite voiture peut passer. On essaie ? La petite voiture rouge attend près du tapis. Toi, tu vas sous le pont. Nino la pousse vers l'arche. Un cube glisse. L'arche a un trou. Oh, elle ne passe pas. Le cube est tombé. Nino repose le cube, trop vite. Le cube penche, de travers. La voiture bute, une seconde fois. Ça ne veut pas ! Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu regardes le cube, d'abord ? Oui, maman. Il pose le cube, sans se presser. L'arche redevient ronde. La voiture passe dessous. Elle est passée ! Elle rentre à la maison ? Oui, puis on s'assoit. Nino veut le t-shirt chaud. Maintenant, le t-shirt ! Il pousse la voiture trop fort. Trois cubes tombent d'un coup. L'arche s'écroule sur la voiture. Oh. Le pont est tombé. Où est ma petite voiture ? Dans la pile de linge ? Nino fouille le t-shirt chaud. Le tissu sent le savon. Pas de voiture. Sous le canapé ? Il se penche. De la poussière, un fil. Elle est perdue. L'éclat de citron tremble, sur le carreau. Je prends tout, d'un coup ! Il saisit la pile trop vite. Les cubes glissent entre ses doigts. Le tapis disparaît sous les cubes. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous les cubes ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>ranger</t>
+          <t>éclat de citron</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,50 +1321,70 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_pont_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le carrelage sent encore le citron.
-narrateur|Papa vient de passer la serpillière.
+          <t>narrateur|L'odeur de citron arrive avant le sol sec.
+narrateur|Papa tord la serpillière au-dessus du seau.
+narrateur|Le seau fait un petit plouf.
+maman|Ça sent le propre.
+papa|Oui, le citron a fini.
+narrateur|Sur un carreau mouillé, un éclat de citron brille.
+enfant-m|Il est jaune, papa.
+papa|C'est le citron, sur le carreau.
 narrateur|Les carreaux sont un peu frais.
 narrateur|Puis le tapis du salon est épais.
-maman|Ça sent le propre.
-papa|Oui, tout propre.
+maman|Le sol est propre, Nino.
+papa|Tu restes sur le tapis ?
+enfant-m|Oui, le sol est mouillé.
 narrateur|Près du canapé, une pile de linge attend.
-narrateur|Un petit t-shirt est encore chaud.
-narrateur|En ce moment, Nino est au milieu du tapis.
-narrateur|Il a des cubes.
-narrateur|Il construit un pont.
-narrateur|Les cubes tapent.
-enfant-m|C'est un pont, papa.
+narrateur|Un petit t-shirt reste chaud, au sommet.
+enfant-m|Je veux mon pont, maintenant !
+maman|Pendant que le sol sèche ?
+enfant-m|Oui, un pont jusqu'au canapé.
+narrateur|En ce moment, Nino saisit un cube.
+narrateur|Le cube bleu pèse un peu, dans sa main.
+narrateur|Il pose le cube sur le tapis épais.
+narrateur|Le bois tape, un petit clic.
+enfant-m|C'est le pont du tapis.
 papa|Un pont bien solide ?
 enfant-m|Oui, il est solide.
 maman|Il va jusqu'où, ton pont ?
 enfant-m|Jusqu'au canapé, maman.
-narrateur|Nino pose encore un cube.
-narrateur|Clic.
-narrateur|Il pose un cube à gauche.
+narrateur|Nino pose un cube à gauche.
 narrateur|Puis un cube à droite.
 narrateur|Le pont a une arche.
 maman|Je vois l'arche, Nino.
 enfant-m|Une petite voiture peut passer.
-papa|On essaie.
-narrateur|Nino prend une petite voiture.
-narrateur|Il la pousse vers l'arche.
+papa|On essaie ?
+narrateur|La petite voiture rouge attend près du tapis.
+enfant-m|Toi, tu vas sous le pont.
+narrateur|Nino la pousse vers l'arche.
 narrateur|Un cube glisse.
 narrateur|L'arche a un trou.
-narrateur|La voiture bute.
 enfant-m|Oh, elle ne passe pas.
 papa|Le cube est tombé.
-narrateur|Nino repose le cube.
-narrateur|Clic.
-narrateur|L'arche est ronde, encore.
+narrateur|Nino repose le cube, trop vite.
+narrateur|Le cube penche, de travers.
+narrateur|La voiture bute, une seconde fois.
+enfant-m|Ça ne veut pas !
+narrateur|Le sourire de Nino disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+maman|Tu regardes le cube, d'abord ?
+enfant-m|Oui, maman.
+narrateur|Il pose le cube, sans se presser.
+narrateur|L'arche redevient ronde.
 narrateur|La voiture passe dessous.
 enfant-m|Elle est passée !
 maman|Elle rentre à la maison ?
 enfant-m|Oui, puis on s'assoit.
 narrateur|Nino veut le t-shirt chaud.
-narrateur|Il pousse encore la voiture.
+enfant-m|Maintenant, le t-shirt !
+narrateur|Il pousse la voiture trop fort.
 narrateur|Trois cubes tombent d'un coup.
 narrateur|L'arche s'écroule sur la voiture.
 enfant-m|Oh.
@@ -1378,12 +1398,20 @@
 narrateur|Il se penche.
 narrateur|De la poussière, un fil.
 enfant-m|Elle est perdue.
-papa|Les cubes sont encore au milieu.
-enfant-m|Je veux voir dessous.
-narrateur|Nino prend un cube.
-narrateur|Il le pose dans la caisse.
-narrateur|Toc.
-narrateur|La caisse sent le bois.</t>
+narrateur|L'éclat de citron tremble, sur le carreau.
+enfant-m|Je prends tout, d'un coup !
+narrateur|Il saisit la pile trop vite.
+narrateur|Les cubes glissent entre ses doigts.
+narrateur|Le tapis disparaît sous les cubes.
+enfant-m|Ça ne veut pas, papa.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu regardes sous les cubes ?</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>serpillière,cubes,voiture</t>
         </is>
       </c>
     </row>
@@ -1415,12 +1443,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nino cherche sa petite voiture. Où est-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nino cherche sa petite &lt;emphasis level="moderate"&gt;voiture&lt;/emphasis&gt;. Où est-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Après le jeu, que fait Martial ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nino cherche sa petite &lt;emphasis&gt;voiture&lt;/emphasis&gt;. Où est-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1483,7 +1511,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1494,7 +1522,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1509,34 +1537,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>voiture</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1551,17 +1583,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=la_voiture_est_sous_les_cubes; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1594,17 +1626,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Un cube de l'arche va dans la caisse. Toc. Tu regardes bien sous le pont ? Oui, maman. Nino écarte un cube à gauche. Un bout de tapis reparaît. Puis un cube à droite. Un toit minuscule brille. Ma voiture ! La petite voiture était sous l'arche. Elle sent encore le bois des cubes. Nino la tient dans la paume. Les roues sont un peu froides. Merci, tu l'as trouvée. Te voilà, petite. Elle était dessous. Les derniers cubes vont dans la caisse. Le tapis devant le canapé est libre. Le t-shirt chaud attend encore.</t>
+          <t>Nino laisse la pile de cubes. Un genou se pose sur le tapis. Sa main trouve un cube bleu. Je le mets, tout seul. Le cube glisse dans la caisse. Toc. Le bois sent un peu le citron. Tu regardes bien dessous ? Oui, maman. Un bout de tapis reparaît. Le cube jaune suit le bleu. Toc. Je sors le reste, d'un coup ! Nino tire trop fort, en bas. Deux cubes retombent, comme un toit. Oh. Cette fois, il ne reprend pas. Il écoute le salon, un instant. Près des cubes, l'éclat de citron brille. Il est là. Nino refuse de foncer. Il écarte un cube, lentement. Un toit minuscule brille. Ma voiture ! La petite voiture était sous l'arche. Elle sent le bois des cubes. Nino la tient dans la paume. Les roues sont un peu froides. Merci, Nino. Elle était dessous. La caisse a presque tous les cubes. Le tapis est libre, au milieu. Le t-shirt peut venir ? Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Un cube de l'arche va dans la caisse. Toc. Tu regardes bien sous le pont ? Oui, maman. Nino écarte un cube à gauche. Un bout de tapis reparaît. Puis un cube à droite. Un toit minuscule brille. Ma voiture ! La petite voiture était sous l'arche. Elle sent encore le bois des cubes. Nino la tient dans la paume. Les roues sont un peu froides. Merci, tu l'as trouvée. Te voilà, petite. Elle était dessous. Les derniers cubes vont dans la caisse. Le tapis devant le canapé est libre. Le t-shirt chaud attend encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino laisse la pile de cubes. Un genou se pose sur le tapis. Sa main trouve un cube bleu. Je le mets, tout seul. Le cube glisse dans la &lt;emphasis level="moderate"&gt;caisse&lt;/emphasis&gt;. Toc. Le bois sent un peu le citron. Tu regardes bien dessous ? Oui, maman. Un bout de tapis reparaît. Le cube jaune suit le bleu. Toc. Je sors le reste, d'un coup ! Nino tire trop fort, en bas. Deux cubes retombent, comme un toit. Oh. Cette fois, il ne reprend pas. Il écoute le salon, un instant. Près des cubes, l'éclat de citron brille. Il est là. Nino refuse de foncer. Il écarte un cube, lentement. Un toit minuscule brille. Ma voiture ! La petite voiture était sous l'arche. Elle sent le bois des cubes. Nino la tient dans la paume. Les roues sont un peu froides. Merci, Nino. Elle était dessous. La caisse a presque tous les cubes. Le tapis est libre, au milieu. Le t-shirt peut venir ? Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Martial a rangé. Les jouets sont dans la &lt;emphasis&gt;caisse&lt;/emphasis&gt;. Le tapis est libre. Papa est là. [pause]</t>
+          <t>Nino laisse la pile de cubes. Un genou se pose sur le tapis. Sa main trouve un cube bleu. Je le mets, tout seul. Le cube glisse dans la &lt;emphasis&gt;caisse&lt;/emphasis&gt;. Toc. Le bois sent un peu le citron. Tu regardes bien dessous ? Oui, maman. Un bout de tapis reparaît. Le cube jaune suit le bleu. Toc. Je sors le reste, d'un coup ! Nino tire trop fort, en bas. Deux cubes retombent, comme un toit. Oh. Cette fois, il ne reprend pas. Il écoute le salon, un instant. Près des cubes, l'éclat de citron brille. Il est là. Nino refuse de foncer. Il écarte un cube, lentement. Un toit minuscule brille. Ma voiture ! La petite voiture était sous l'arche. Elle sent le bois des cubes. Nino la tient dans la paume. Les roues sont un peu froides. Merci, Nino. Elle était dessous. La caisse a presque tous les cubes. Le tapis est libre, au milieu. Le t-shirt peut venir ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1651,7 +1683,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1659,10 +1691,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1692,23 +1724,23 @@
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1717,10 +1749,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1733,30 +1765,50 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_pose_un_cube_sans_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Un cube de l'arche va dans la caisse.
+          <t>narrateur|Nino laisse la pile de cubes.
+narrateur|Un genou se pose sur le tapis.
+narrateur|Sa main trouve un cube bleu.
+enfant-m|Je le mets, tout seul.
+narrateur|Le cube glisse dans la caisse.
 narrateur|Toc.
-maman|Tu regardes bien sous le pont ?
+narrateur|Le bois sent un peu le citron.
+maman|Tu regardes bien dessous ?
 enfant-m|Oui, maman.
-narrateur|Nino écarte un cube à gauche.
-papa|Un bout de tapis reparaît.
-narrateur|Puis un cube à droite.
+narrateur|Un bout de tapis reparaît.
+narrateur|Le cube jaune suit le bleu.
+narrateur|Toc.
+enfant-m|Je sors le reste, d'un coup !
+narrateur|Nino tire trop fort, en bas.
+narrateur|Deux cubes retombent, comme un toit.
+enfant-m|Oh.
+narrateur|Cette fois, il ne reprend pas.
+narrateur|Il écoute le salon, un instant.
+narrateur|Près des cubes, l'éclat de citron brille.
+enfant-m|Il est là.
+narrateur|Nino refuse de foncer.
+narrateur|Il écarte un cube, lentement.
 narrateur|Un toit minuscule brille.
 enfant-m|Ma voiture !
 narrateur|La petite voiture était sous l'arche.
-narrateur|Elle sent encore le bois des cubes.
+narrateur|Elle sent le bois des cubes.
 narrateur|Nino la tient dans la paume.
 narrateur|Les roues sont un peu froides.
-papa|Merci, tu l'as trouvée.
-maman|Te voilà, petite.
+papa|Merci, Nino.
 enfant-m|Elle était dessous.
-narrateur|Les derniers cubes vont dans la caisse.
-narrateur|Le tapis devant le canapé est libre.
-narrateur|Le t-shirt chaud attend encore.</t>
+narrateur|La caisse a presque tous les cubes.
+narrateur|Le tapis est libre, au milieu.
+maman|Le t-shirt peut venir ?
+enfant-m|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>caisse,bois</t>
         </is>
       </c>
     </row>
@@ -1783,17 +1835,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nino pousse la caisse sous la table. Le bois glisse un peu. Le t-shirt, maintenant ? Oui, il est chaud. Maman lui tend le t-shirt. Nino l'enfile. Le tissu sent le savon, tout chaud. On s'assoit ? Oui, papa. Nino grimpe sur le canapé. La petite voiture est sur ses genoux. Tu veux un verre d'eau ? Oui, maman. L'eau est fraîche, après le citron. Nino boit une gorgée. Le pont a fini sa journée. La voiture aussi. La pile de linge reste douce, près d'eux.</t>
+          <t>On prend le t-shirt ? Nino va vers la pile tiède. Je prends tout ! Il tire trop fort sur le tas. Une chaussette tombe, molle. Oh. Nino s'arrête net. Il refuse de foncer. Attends, je regarde. Il prend le t-shirt, seul. Il est chaud, celui-là. Oui, maman. Maman lui tend le tissu. Nino l'enfile. Le tissu sent le savon, bien chaud. La caisse, Nino ? Je la pousse. Nino pousse la caisse près du canapé. Le bois glisse un peu. On s'assoit ? Oui, papa. Nino grimpe sur le canapé. La petite voiture est sur ses genoux. Tu veux un verre d'eau ? Oui, maman. L'eau est fraîche, après le citron. Nino boit une gorgée. Le pont a fini sa journée. La voiture aussi.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nino pousse la caisse sous la table. Le bois glisse un peu. Le t-shirt, maintenant ? Oui, il est chaud. Maman lui tend le t-shirt. Nino l'enfile. Le tissu sent le savon, tout chaud. On s'assoit ? Oui, papa. Nino grimpe sur le canapé. La petite voiture est sur ses genoux. Tu veux un verre d'eau ? Oui, maman. L'eau est fraîche, après le citron. Nino boit une gorgée. Le pont a fini sa journée. La voiture aussi. La pile de linge reste douce, près d'eux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On prend le &lt;emphasis level="moderate"&gt;t-shirt&lt;/emphasis&gt; ? Nino va vers la pile tiède. Je prends tout ! Il tire trop fort sur le tas. Une chaussette tombe, molle. Oh. Nino s'arrête net. Il refuse de foncer. Attends, je regarde. Il prend le t-shirt, seul. Il est chaud, celui-là. Oui, maman. Maman lui tend le tissu. Nino l'enfile. Le tissu sent le savon, bien chaud. La caisse, Nino ? Je la pousse. Nino pousse la caisse près du canapé. Le bois glisse un peu. On s'assoit ? Oui, papa. Nino grimpe sur le canapé. La petite voiture est sur ses genoux. Tu veux un verre d'eau ? Oui, maman. L'eau est fraîche, après le citron. Nino boit une gorgée. Le pont a fini sa journée. La voiture aussi.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Martial pousse la &lt;emphasis&gt;caisse&lt;/emphasis&gt; sous la table. Papa tend un verre d'eau. [pause]</t>
+          <t>On prend le &lt;emphasis&gt;t-shirt&lt;/emphasis&gt; ? Nino va vers la pile tiède. Je prends tout ! Il tire trop fort sur le tas. Une chaussette tombe, molle. Oh. Nino s'arrête net. Il refuse de foncer. Attends, je regarde. Il prend le t-shirt, seul. Il est chaud, celui-là. Oui, maman. Maman lui tend le tissu. Nino l'enfile. Le tissu sent le savon, bien chaud. La caisse, Nino ? Je la pousse. Nino pousse la caisse près du canapé. Le bois glisse un peu. On s'assoit ? Oui, papa. Nino grimpe sur le canapé. La petite voiture est sur ses genoux. Tu veux un verre d'eau ? Oui, maman. L'eau est fraîche, après le citron. Nino boit une gorgée. Le pont a fini sa journée. La voiture aussi. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1840,7 +1892,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1848,10 +1900,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1874,30 +1926,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>caisse</t>
+          <t>t-shirt</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1906,10 +1958,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1920,16 +1972,32 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_tirer_toute_la_pile; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nino pousse la caisse sous la table.
+          <t>papa|On prend le t-shirt ?
+narrateur|Nino va vers la pile tiède.
+enfant-m|Je prends tout !
+narrateur|Il tire trop fort sur le tas.
+narrateur|Une chaussette tombe, molle.
+enfant-m|Oh.
+narrateur|Nino s'arrête net.
+narrateur|Il refuse de foncer.
+enfant-m|Attends, je regarde.
+narrateur|Il prend le t-shirt, seul.
+maman|Il est chaud, celui-là.
+enfant-m|Oui, maman.
+narrateur|Maman lui tend le tissu.
+narrateur|Nino l'enfile.
+narrateur|Le tissu sent le savon, bien chaud.
+papa|La caisse, Nino ?
+enfant-m|Je la pousse.
+narrateur|Nino pousse la caisse près du canapé.
 narrateur|Le bois glisse un peu.
-maman|Le t-shirt, maintenant ?
-enfant-m|Oui, il est chaud.
-narrateur|Maman lui tend le t-shirt.
-narrateur|Nino l'enfile.
-narrateur|Le tissu sent le savon, tout chaud.
 papa|On s'assoit ?
 enfant-m|Oui, papa.
 narrateur|Nino grimpe sur le canapé.
@@ -1939,8 +2007,12 @@
 narrateur|L'eau est fraîche, après le citron.
 narrateur|Nino boit une gorgée.
 papa|Le pont a fini sa journée.
-enfant-m|La voiture aussi.
-narrateur|La pile de linge reste douce, près d'eux.</t>
+enfant-m|La voiture aussi.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>linge,canapé</t>
         </is>
       </c>
     </row>
@@ -1967,17 +2039,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La voiture est sur mes genoux. Toi aussi, tu es au chaud. Bravo, tu l'as retrouvée. Le t-shirt garde encore la chaleur. Le citron du carrelage s'en va, tout doux.</t>
+          <t>Ils s'assoient près de la pile tiède. La chaleur touche les joues de Nino. La voiture est sur mes genoux. Toi aussi, tu es au chaud. Comme sur le carreau, papa ! Tu le vois, toi ? Oui, le petit jaune. Nino glisse la voiture sans se presser. Le métal repose contre sa hanche. On le sent, maman. Tu le sens sur tes joues ? Oui, il est chaud. Le carreau est libre, Nino. Comme au début, papa. Le citron reste dans l'air. L'éclat de citron tient sur le carreau.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La voiture est sur mes genoux. Toi aussi, tu es au chaud. Bravo, tu l'as retrouvée. Le t-shirt garde encore la chaleur. Le citron du carrelage s'en va, tout doux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils s'assoient près de la pile tiède. La chaleur touche les joues de Nino. La voiture est sur mes genoux. Toi aussi, tu es au chaud. Comme sur le carreau, papa ! Tu le vois, toi ? Oui, le petit jaune. Nino glisse la voiture sans se presser. Le métal repose contre sa hanche. On le sent, maman. Tu le sens sur tes joues ? Oui, il est chaud. Le carreau est libre, Nino. Comme au début, papa. Le citron reste dans l'air. L'&lt;emphasis level="moderate"&gt;éclat de citron&lt;/emphasis&gt; tient sur le carreau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils s'assoient près de la pile tiède. La chaleur touche les joues de Nino. La voiture est sur mes genoux. Toi aussi, tu es au chaud. Comme sur le carreau, papa ! Tu le vois, toi ? Oui, le petit jaune. Nino glisse la voiture sans se presser. Le métal repose contre sa hanche. On le sent, maman. Tu le sens sur tes joues ? Oui, il est chaud. Le carreau est libre, Nino. Comme au début, papa. Le citron reste dans l'air. L'&lt;emphasis&gt;éclat de citron&lt;/emphasis&gt; tient sur le carreau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2024,18 +2096,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2044,12 +2116,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2058,17 +2130,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de citron</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2077,11 +2153,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2090,28 +2166,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_carreau; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|La voiture est sur mes genoux.
+          <t>narrateur|Ils s'assoient près de la pile tiède.
+narrateur|La chaleur touche les joues de Nino.
+enfant-m|La voiture est sur mes genoux.
 maman|Toi aussi, tu es au chaud.
-papa|Bravo, tu l'as retrouvée.
-narrateur|Le t-shirt garde encore la chaleur.
-narrateur|Le citron du carrelage s'en va, tout doux.</t>
+enfant-m|Comme sur le carreau, papa !
+papa|Tu le vois, toi ?
+enfant-m|Oui, le petit jaune.
+narrateur|Nino glisse la voiture sans se presser.
+narrateur|Le métal repose contre sa hanche.
+enfant-m|On le sent, maman.
+maman|Tu le sens sur tes joues ?
+enfant-m|Oui, il est chaud.
+papa|Le carreau est libre, Nino.
+enfant-m|Comme au début, papa.
+narrateur|Le citron reste dans l'air.
+narrateur|L'éclat de citron tient sur le carreau.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>citron,canapé</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2224,6 +2320,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>